<commit_message>
fix(lead-magnet): fix ROUND formula syntax in Sheet1 ROI calculation column
</commit_message>
<xml_diff>
--- a/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
+++ b/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="H4" s="17">
-        <f>IF(G4="","",ROUND((VALUE(LEFT(E4,1))*0.5+VALUE(LEFT(F4,1))*0.3+IF(LEFT(G4,1)="H",1,IF(LEFT(G4,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G4="","",ROUND(VALUE(LEFT(E4,1))*0.5+VALUE(LEFT(F4,1))*0.3+IF(LEFT(G4,1)="H",1,IF(LEFT(G4,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="H5" s="17">
-        <f>IF(G5="","",ROUND((VALUE(LEFT(E5,1))*0.5+VALUE(LEFT(F5,1))*0.3+IF(LEFT(G5,1)="H",1,IF(LEFT(G5,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G5="","",ROUND(VALUE(LEFT(E5,1))*0.5+VALUE(LEFT(F5,1))*0.3+IF(LEFT(G5,1)="H",1,IF(LEFT(G5,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       <c r="F6" s="18" t="inlineStr"/>
       <c r="G6" s="18" t="inlineStr"/>
       <c r="H6" s="17">
-        <f>IF(G6="","",ROUND((VALUE(LEFT(E6,1))*0.5+VALUE(LEFT(F6,1))*0.3+IF(LEFT(G6,1)="H",1,IF(LEFT(G6,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G6="","",ROUND(VALUE(LEFT(E6,1))*0.5+VALUE(LEFT(F6,1))*0.3+IF(LEFT(G6,1)="H",1,IF(LEFT(G6,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       <c r="F7" s="18" t="inlineStr"/>
       <c r="G7" s="18" t="inlineStr"/>
       <c r="H7" s="17">
-        <f>IF(G7="","",ROUND((VALUE(LEFT(E7,1))*0.5+VALUE(LEFT(F7,1))*0.3+IF(LEFT(G7,1)="H",1,IF(LEFT(G7,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G7="","",ROUND(VALUE(LEFT(E7,1))*0.5+VALUE(LEFT(F7,1))*0.3+IF(LEFT(G7,1)="H",1,IF(LEFT(G7,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       <c r="F8" s="18" t="inlineStr"/>
       <c r="G8" s="18" t="inlineStr"/>
       <c r="H8" s="17">
-        <f>IF(G8="","",ROUND((VALUE(LEFT(E8,1))*0.5+VALUE(LEFT(F8,1))*0.3+IF(LEFT(G8,1)="H",1,IF(LEFT(G8,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G8="","",ROUND(VALUE(LEFT(E8,1))*0.5+VALUE(LEFT(F8,1))*0.3+IF(LEFT(G8,1)="H",1,IF(LEFT(G8,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       <c r="F9" s="18" t="inlineStr"/>
       <c r="G9" s="18" t="inlineStr"/>
       <c r="H9" s="17">
-        <f>IF(G9="","",ROUND((VALUE(LEFT(E9,1))*0.5+VALUE(LEFT(F9,1))*0.3+IF(LEFT(G9,1)="H",1,IF(LEFT(G9,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G9="","",ROUND(VALUE(LEFT(E9,1))*0.5+VALUE(LEFT(F9,1))*0.3+IF(LEFT(G9,1)="H",1,IF(LEFT(G9,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       <c r="F10" s="18" t="inlineStr"/>
       <c r="G10" s="18" t="inlineStr"/>
       <c r="H10" s="17">
-        <f>IF(G10="","",ROUND((VALUE(LEFT(E10,1))*0.5+VALUE(LEFT(F10,1))*0.3+IF(LEFT(G10,1)="H",1,IF(LEFT(G10,1)="M",3,5))*0.2)*10)/10)</f>
+        <f>IF(G10="","",ROUND(VALUE(LEFT(E10,1))*0.5+VALUE(LEFT(F10,1))*0.3+IF(LEFT(G10,1)="H",1,IF(LEFT(G10,1)="M",3,5))*0.2,1))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: repair structural XML metadata in phoenix_ai_canvas_4plus1.xlsx by resaving with openpyxl
</commit_message>
<xml_diff>
--- a/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
+++ b/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
@@ -158,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -236,11 +236,287 @@
         <color rgb="00BDC3C7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="006E2F8A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="006E2F8A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="006E2F8A"/>
+      </right>
+      <top style="medium">
+        <color rgb="006E2F8A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="006E2F8A"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="006E2F8A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="006E2F8A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="006E2F8A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="006E2F8A"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="006E2F8A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B4F72"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B4F72"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B4F72"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B4F72"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B4F72"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B4F72"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B4F72"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B4F72"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B4F72"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B4F72"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="007D3C14"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="007D3C14"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="007D3C14"/>
+      </right>
+      <top style="medium">
+        <color rgb="007D3C14"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="007D3C14"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="007D3C14"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="007D3C14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="007D3C14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="007D3C14"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="007D3C14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00145A32"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00145A32"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00145A32"/>
+      </right>
+      <top style="medium">
+        <color rgb="00145A32"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00145A32"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00145A32"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00145A32"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00145A32"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00145A32"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00145A32"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -326,6 +602,34 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -748,6 +1052,9 @@
 ▪ 試點場景名稱：</t>
         </is>
       </c>
+      <c r="B5" s="29" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="30" t="n"/>
       <c r="E5" s="7" t="inlineStr">
         <is>
           <t>▪ 技術路徑（SaaS/API/私有化）：
@@ -756,6 +1063,9 @@
 ▪ 上線預計時程：</t>
         </is>
       </c>
+      <c r="F5" s="31" t="n"/>
+      <c r="G5" s="31" t="n"/>
+      <c r="H5" s="32" t="n"/>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>▪ 核心資料來源與格式：
@@ -764,13 +1074,64 @@
 ▪ 第三道防線（審計日誌）：</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1"/>
-    <row r="7" ht="22" customHeight="1"/>
-    <row r="8" ht="22" customHeight="1"/>
-    <row r="9" ht="22" customHeight="1"/>
-    <row r="10" ht="22" customHeight="1"/>
-    <row r="11" ht="22" customHeight="1"/>
+      <c r="J5" s="33" t="n"/>
+      <c r="K5" s="33" t="n"/>
+      <c r="L5" s="34" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="35" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="37" t="n"/>
+      <c r="H6" s="38" t="n"/>
+      <c r="I6" s="39" t="n"/>
+      <c r="L6" s="40" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="35" t="n"/>
+      <c r="D7" s="36" t="n"/>
+      <c r="E7" s="37" t="n"/>
+      <c r="H7" s="38" t="n"/>
+      <c r="I7" s="39" t="n"/>
+      <c r="L7" s="40" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="35" t="n"/>
+      <c r="D8" s="36" t="n"/>
+      <c r="E8" s="37" t="n"/>
+      <c r="H8" s="38" t="n"/>
+      <c r="I8" s="39" t="n"/>
+      <c r="L8" s="40" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="35" t="n"/>
+      <c r="D9" s="36" t="n"/>
+      <c r="E9" s="37" t="n"/>
+      <c r="H9" s="38" t="n"/>
+      <c r="I9" s="39" t="n"/>
+      <c r="L9" s="40" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="35" t="n"/>
+      <c r="D10" s="36" t="n"/>
+      <c r="E10" s="37" t="n"/>
+      <c r="H10" s="38" t="n"/>
+      <c r="I10" s="39" t="n"/>
+      <c r="L10" s="40" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="41" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="42" t="n"/>
+      <c r="D11" s="43" t="n"/>
+      <c r="E11" s="44" t="n"/>
+      <c r="F11" s="45" t="n"/>
+      <c r="G11" s="45" t="n"/>
+      <c r="H11" s="46" t="n"/>
+      <c r="I11" s="47" t="n"/>
+      <c r="J11" s="48" t="n"/>
+      <c r="K11" s="48" t="n"/>
+      <c r="L11" s="49" t="n"/>
+    </row>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -798,6 +1159,9 @@
 ▪ 擴展複製路徑：</t>
         </is>
       </c>
+      <c r="B14" s="29" t="n"/>
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="30" t="n"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
           <t>▪ 一線員工核心阻力：
@@ -806,6 +1170,9 @@
 ▪ 技能培訓計畫：</t>
         </is>
       </c>
+      <c r="F14" s="33" t="n"/>
+      <c r="G14" s="33" t="n"/>
+      <c r="H14" s="34" t="n"/>
       <c r="I14" s="10" t="inlineStr">
         <is>
           <t>▪ 人機決策分工（HITL）：
@@ -814,13 +1181,64 @@
 ▪ ISO 42001 稽核計畫：</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="22" customHeight="1"/>
-    <row r="16" ht="22" customHeight="1"/>
-    <row r="17" ht="22" customHeight="1"/>
-    <row r="18" ht="22" customHeight="1"/>
-    <row r="19" ht="22" customHeight="1"/>
-    <row r="20" ht="22" customHeight="1"/>
+      <c r="J14" s="50" t="n"/>
+      <c r="K14" s="50" t="n"/>
+      <c r="L14" s="51" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="35" t="n"/>
+      <c r="D15" s="36" t="n"/>
+      <c r="E15" s="39" t="n"/>
+      <c r="H15" s="40" t="n"/>
+      <c r="I15" s="52" t="n"/>
+      <c r="L15" s="53" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="35" t="n"/>
+      <c r="D16" s="36" t="n"/>
+      <c r="E16" s="39" t="n"/>
+      <c r="H16" s="40" t="n"/>
+      <c r="I16" s="52" t="n"/>
+      <c r="L16" s="53" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="35" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="39" t="n"/>
+      <c r="H17" s="40" t="n"/>
+      <c r="I17" s="52" t="n"/>
+      <c r="L17" s="53" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="35" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="39" t="n"/>
+      <c r="H18" s="40" t="n"/>
+      <c r="I18" s="52" t="n"/>
+      <c r="L18" s="53" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="35" t="n"/>
+      <c r="D19" s="36" t="n"/>
+      <c r="E19" s="39" t="n"/>
+      <c r="H19" s="40" t="n"/>
+      <c r="I19" s="52" t="n"/>
+      <c r="L19" s="53" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="41" t="n"/>
+      <c r="B20" s="42" t="n"/>
+      <c r="C20" s="42" t="n"/>
+      <c r="D20" s="43" t="n"/>
+      <c r="E20" s="47" t="n"/>
+      <c r="F20" s="48" t="n"/>
+      <c r="G20" s="48" t="n"/>
+      <c r="H20" s="49" t="n"/>
+      <c r="I20" s="54" t="n"/>
+      <c r="J20" s="55" t="n"/>
+      <c r="K20" s="55" t="n"/>
+      <c r="L20" s="56" t="n"/>
+    </row>
     <row r="21" ht="22" customHeight="1"/>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="11" t="inlineStr">

</xml_diff>

<commit_message>
fix: rename sheet names in phoenix_ai_canvas_4plus1.xlsx to remove emojis and colons to prevent Excel load warning
</commit_message>
<xml_diff>
--- a/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
+++ b/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="👑 總表：一頁式戰略畫布" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📋 主表一：場景盤點" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="📋 主表二：架構與資安" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📋 主表三：試點與變革" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="📋 主表四：營運與治理" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="總表-一頁式戰略畫布" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="主表一-場景盤點" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="主表二-架構與資安" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="主表三-試點與變革" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="主表四-營運與治理" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: design and add AI Video Tools Selection and Financial Diagnostics sheet as Sheet 7 of strategy canvas
</commit_message>
<xml_diff>
--- a/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
+++ b/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
@@ -12,7 +12,8 @@
     <sheet name="主表二-架構與資安" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="主表三-試點與變革" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="附表-RAG採購5維自診" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="主表四-營運與治理" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="附表-影片工具選型與財務自診" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="主表四-營運與治理" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -270,7 +271,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -718,11 +719,44 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -896,6 +930,7 @@
     <xf numFmtId="0" fontId="19" fillId="23" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -2291,11 +2326,6 @@
           <t>📋 附表：企業 RAG 採購與數據成熟度 5 維自評表 (RAG Procurement &amp; Data Readiness Diagnostics)</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
     </row>
     <row r="2" ht="35" customHeight="1" s="12">
       <c r="A2" s="73" t="inlineStr">
@@ -2303,11 +2333,6 @@
           <t xml:space="preserve">  ℹ️ 使用說明：本表為 RAG 企業級知識庫採購前的自我成熟度評估表。請針對以下 5 個維度進行自評打分 (每項 1~5 分)，總分將會自動加總，並出具對應的顧問落地路徑診斷與避坑指南。</t>
         </is>
       </c>
-      <c r="B2" s="74" t="n"/>
-      <c r="C2" s="74" t="n"/>
-      <c r="D2" s="74" t="n"/>
-      <c r="E2" s="74" t="n"/>
-      <c r="F2" s="74" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1" s="12">
       <c r="A3" s="75" t="inlineStr">
@@ -2492,7 +2517,7 @@
           <t>📈 成熟度診斷結果：</t>
         </is>
       </c>
-      <c r="B9" s="79" t="n"/>
+      <c r="B9" s="83" t="n"/>
       <c r="C9" s="80" t="inlineStr">
         <is>
           <t>🤖 總分自評加總：</t>
@@ -2506,7 +2531,7 @@
         <f>IF(D9&lt;=12,"🔴 警訊：基礎建設薄弱。建議首要做數據清洗，暫緩軟體採購，防範高額黑洞。",IF(D9&lt;=19,"🟡 建議：採用 SaaS/API 混合架構，並配置嚴格的「真人雙簽 (HITL)」防線。","🟢 優勢：就緒度高。可自建或深度客製化 RAG 系統，直接開展試點。"))</f>
         <v/>
       </c>
-      <c r="F9" s="79" t="n"/>
+      <c r="F9" s="83" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2520,6 +2545,286 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="12" min="1" max="1"/>
+    <col width="24" customWidth="1" style="12" min="2" max="2"/>
+    <col width="45" customWidth="1" style="12" min="3" max="3"/>
+    <col width="16" customWidth="1" style="12" min="4" max="4"/>
+    <col width="50" customWidth="1" style="12" min="5" max="5"/>
+    <col width="30" customWidth="1" style="12" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1" s="12">
+      <c r="A1" s="71" t="inlineStr">
+        <is>
+          <t>📋 附表：商用行銷影片 6 大工具選型與財務自診表 (AI Video Tools Selection &amp; Financial Diagnostics)</t>
+        </is>
+      </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+    </row>
+    <row r="2" ht="35" customHeight="1" s="12">
+      <c r="A2" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ℹ️ 使用說明：本表供企業在採購或導入 AI 行銷影片生成工具 (如 Sora, Kling, Runway, HeyGen) 前進行評估。請針對以下 6 個維度進行自評打分 (每項 1~5 分)，以診斷工具的商用合規度、Token 財務 TCO 成本與特徵一致性就緒度。</t>
+        </is>
+      </c>
+      <c r="B2" s="74" t="n"/>
+      <c r="C2" s="74" t="n"/>
+      <c r="D2" s="74" t="n"/>
+      <c r="E2" s="74" t="n"/>
+      <c r="F2" s="74" t="n"/>
+    </row>
+    <row r="3" ht="25" customHeight="1" s="12">
+      <c r="A3" s="75" t="inlineStr">
+        <is>
+          <t>評估維度</t>
+        </is>
+      </c>
+      <c r="B3" s="75" t="inlineStr">
+        <is>
+          <t>自評項目</t>
+        </is>
+      </c>
+      <c r="C3" s="75" t="inlineStr">
+        <is>
+          <t>指標說明</t>
+        </is>
+      </c>
+      <c r="D3" s="75" t="inlineStr">
+        <is>
+          <t>自評分數 (1-5)</t>
+        </is>
+      </c>
+      <c r="E3" s="75" t="inlineStr">
+        <is>
+          <t>選型評估與財務指引</t>
+        </is>
+      </c>
+      <c r="F3" s="75" t="inlineStr">
+        <is>
+          <t>備註 / 企業現況</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1" s="12">
+      <c r="A4" s="76" t="inlineStr">
+        <is>
+          <t>維度一：肖像權合規風險</t>
+        </is>
+      </c>
+      <c r="B4" s="76" t="inlineStr">
+        <is>
+          <t>肖像權合規風險
+(商用免責承諾)</t>
+        </is>
+      </c>
+      <c r="C4" s="77" t="inlineStr">
+        <is>
+          <t>評估工具生成的虛擬人物或聲音是否會侵犯第三方肖像權或著作權，以及平台是否提供 B2B 客戶商用版權免責保護。</t>
+        </is>
+      </c>
+      <c r="D4" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="77" t="inlineStr">
+        <is>
+          <t>1 分：開源或免費版，無任何授權保證，面臨高度侵權與客訴風險
+3 分：有付費套餐，但合約中無明確的智慧財產權商用免責保護條款
+5 分：企業級 SaaS，正式合約條款中明文承諾「商用安全免責保障」</t>
+        </is>
+      </c>
+      <c r="F4" s="77" t="inlineStr"/>
+    </row>
+    <row r="5" ht="60" customHeight="1" s="12">
+      <c r="A5" s="76" t="inlineStr">
+        <is>
+          <t>維度二：TCO 算力財務控制</t>
+        </is>
+      </c>
+      <c r="B5" s="76" t="inlineStr">
+        <is>
+          <t>Token 算力財務 TCO 控制
+(點數消耗與費用限制)</t>
+        </is>
+      </c>
+      <c r="C5" s="77" t="inlineStr">
+        <is>
+          <t>影片生成算力消耗巨大，需要精算單次生成成本 (點數消耗率) 及企業整體的預算控制與防超付機制。</t>
+        </is>
+      </c>
+      <c r="D5" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="77" t="inlineStr">
+        <is>
+          <t>1 分：單次生成成本極高，疊代修改費用昂貴，且缺乏預算限制功能
+3 分：提供基本套餐點數，但多版本修改容易超出額度，費用較高
+5 分：具備算力優化技術，單次消耗點數低，且具備部門限額管理</t>
+        </is>
+      </c>
+      <c r="F5" s="77" t="inlineStr"/>
+    </row>
+    <row r="6" ht="60" customHeight="1" s="12">
+      <c r="A6" s="76" t="inlineStr">
+        <is>
+          <t>維度三：品牌聲調對齊度</t>
+        </is>
+      </c>
+      <c r="B6" s="76" t="inlineStr">
+        <is>
+          <t>品牌聲調 DPO 對齊度
+(自建 Prompt 路由)</t>
+        </is>
+      </c>
+      <c r="C6" s="77" t="inlineStr">
+        <is>
+          <t>影片整體風格、旁白配音與品牌調性的對齊程度。是否能接回內部 Prompt 路由器進行統一控管。</t>
+        </is>
+      </c>
+      <c r="D6" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="77" t="inlineStr">
+        <is>
+          <t>1 分：僅能套用固定模板，配音生硬且無法對齊品牌形象調性
+3 分：支援自定義 Prompt 輸入，但風格無法精細對齊，仍需手動微調
+5 分：支援企業語音克隆與專屬 DPO 對齊，可無縫串接 Router Prompt</t>
+        </is>
+      </c>
+      <c r="F6" s="77" t="inlineStr"/>
+    </row>
+    <row r="7" ht="60" customHeight="1" s="12">
+      <c r="A7" s="76" t="inlineStr">
+        <is>
+          <t>維度四：物理特徵一致性</t>
+        </is>
+      </c>
+      <c r="B7" s="76" t="inlineStr">
+        <is>
+          <t>物理特徵一致性
+(LOGO與產品渲染精準度)</t>
+        </is>
+      </c>
+      <c r="C7" s="77" t="inlineStr">
+        <is>
+          <t>評估影片中「產品細節、企業 LOGO、主角面部」在不同鏡頭切換間的一致性，防止影片產生扭曲變形等穿幫畫面。</t>
+        </is>
+      </c>
+      <c r="D7" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="77" t="inlineStr">
+        <is>
+          <t>1 分：每秒畫面穿幫嚴重，LOGO 或產品細節在每幀快速變形扭曲
+3 分：主體畫面一致，但在大角度或快速運鏡時細節仍會失真穿幫
+5 分：支援 Reference Frame 或 3D 模型導入，特徵一致性達 98%</t>
+        </is>
+      </c>
+      <c r="F7" s="77" t="inlineStr"/>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="12">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>維度五：口型與語音克隆</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>多國口型與語音克隆對齊
+(外銷口型同步)</t>
+        </is>
+      </c>
+      <c r="C8" s="77" t="inlineStr">
+        <is>
+          <t>針對外銷多語系影片，評估 AI 生成的翻譯語音與畫面中人物口型的對齊精準度，避免不自然的視覺違和感。</t>
+        </is>
+      </c>
+      <c r="D8" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="77" t="inlineStr">
+        <is>
+          <t>1 分：配音腔調極不自然且口型完全對不上，視覺違和感重
+3 分：支援多國配音，但口型同步率中等，有輕微滯後感
+5 分：具備高精度語音克隆 (Voice Cloning) 與 AI 口型對齊 (Lip-sync)</t>
+        </is>
+      </c>
+      <c r="F8" s="77" t="inlineStr"/>
+    </row>
+    <row r="9" ht="60" customHeight="1" s="12">
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>維度六：本地剪輯工具對接</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>非侵入式本地剪輯對接
+(剪輯工作流與著作權)</t>
+        </is>
+      </c>
+      <c r="C9" s="77" t="inlineStr">
+        <is>
+          <t>評估 AI 生成素材是否能與現有剪輯軟體 (Premiere/CapCut) 無縫整合，以及生成素材的版權歸屬保障。</t>
+        </is>
+      </c>
+      <c r="D9" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="77" t="inlineStr">
+        <is>
+          <t>1 分：全網頁操作，無法與本地剪輯工作流連動，生成版權不明確
+3 分：可導出標準 MP4，但缺乏 API 支援，需手動下載與導入剪輯
+5 分：提供完整的 API 接口，支援本地自動化剪輯，素材產權歸屬企業</t>
+        </is>
+      </c>
+      <c r="F9" s="77" t="inlineStr"/>
+    </row>
+    <row r="10" ht="45" customHeight="1" s="12">
+      <c r="A10" s="78" t="inlineStr">
+        <is>
+          <t>📈 選型財務診斷結果：</t>
+        </is>
+      </c>
+      <c r="B10" s="79" t="n"/>
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t>🤖 總分自評加總：</t>
+        </is>
+      </c>
+      <c r="D10" s="81">
+        <f>SUM(D4:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="82">
+        <f>IF(D10&lt;=15,"🔴 警訊：預算或技術一致性不足。不建議盲目採購高階 SaaS 專案，應先以小範圍免費工具驗證。",IF(D10&lt;=23,"🟡 建議：採用 2/8 原則。使用 SaaS 進行草稿生成，並由一線剪輯師進行人機協作 (HITL) 覆核修剪。","🟢 優勢：就緒度高。可大規模採購 API 或企業級 SaaS，建立全自動行銷影片製作流水線。"))</f>
+        <v/>
+      </c>
+      <c r="F10" s="79" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A10:B10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat: Add '員工AI肖像授權' sheet (Sheet 8) to strategy canvas
</commit_message>
<xml_diff>
--- a/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
+++ b/curriculum/unit_7_strategy/phoenix_ai_canvas_4plus1.xlsx
@@ -13,7 +13,8 @@
     <sheet name="主表三-試點與變革" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="附表-RAG採購5維自診" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="附表-影片工具選型與財務自診" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="主表四-營運與治理" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="附表-員工AI肖像授權" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="主表四-營運與治理" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="27">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -143,8 +144,40 @@
       <color rgb="00FF5B35"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <i val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="24">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -270,8 +303,14 @@
         <bgColor rgb="00FCF3CF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="45">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -752,11 +791,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -931,6 +976,27 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -2567,11 +2633,6 @@
           <t>📋 附表：商用行銷影片 6 大工具選型與財務自診表 (AI Video Tools Selection &amp; Financial Diagnostics)</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
     </row>
     <row r="2" ht="35" customHeight="1" s="12">
       <c r="A2" s="73" t="inlineStr">
@@ -2579,11 +2640,6 @@
           <t xml:space="preserve">  ℹ️ 使用說明：本表供企業在採購或導入 AI 行銷影片生成工具 (如 Sora, Kling, Runway, HeyGen) 前進行評估。請針對以下 6 個維度進行自評打分 (每項 1~5 分)，以診斷工具的商用合規度、Token 財務 TCO 成本與特徵一致性就緒度。</t>
         </is>
       </c>
-      <c r="B2" s="74" t="n"/>
-      <c r="C2" s="74" t="n"/>
-      <c r="D2" s="74" t="n"/>
-      <c r="E2" s="74" t="n"/>
-      <c r="F2" s="74" t="n"/>
     </row>
     <row r="3" ht="25" customHeight="1" s="12">
       <c r="A3" s="75" t="inlineStr">
@@ -2797,7 +2853,7 @@
           <t>📈 選型財務診斷結果：</t>
         </is>
       </c>
-      <c r="B10" s="79" t="n"/>
+      <c r="B10" s="83" t="n"/>
       <c r="C10" s="80" t="inlineStr">
         <is>
           <t>🤖 總分自評加總：</t>
@@ -2811,7 +2867,7 @@
         <f>IF(D10&lt;=15,"🔴 警訊：預算或技術一致性不足。不建議盲目採購高階 SaaS 專案，應先以小範圍免費工具驗證。",IF(D10&lt;=23,"🟡 建議：採用 2/8 原則。使用 SaaS 進行草稿生成，並由一線剪輯師進行人機協作 (HITL) 覆核修剪。","🟢 優勢：就緒度高。可大規模採購 API 或企業級 SaaS，建立全自動行銷影片製作流水線。"))</f>
         <v/>
       </c>
-      <c r="F10" s="79" t="n"/>
+      <c r="F10" s="83" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2825,6 +2881,140 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="12" min="1" max="1"/>
+    <col width="50" customWidth="1" style="12" min="2" max="2"/>
+    <col width="50" customWidth="1" style="12" min="3" max="3"/>
+    <col width="25" customWidth="1" style="12" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="12">
+      <c r="A1" s="84" t="inlineStr">
+        <is>
+          <t>員工 AI 肖像永久商用授權同意書 (對照自診與修改草案)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="85" t="inlineStr">
+        <is>
+          <t>評估貴公司目前的合約是否有涵蓋這三個保命條款，避免產生肖像侵權爭議。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1" s="12">
+      <c r="A3" s="86" t="inlineStr">
+        <is>
+          <t>條款類型</t>
+        </is>
+      </c>
+      <c r="B3" s="86" t="inlineStr">
+        <is>
+          <t>NG 合約寫法 (潛在風險)</t>
+        </is>
+      </c>
+      <c r="C3" s="86" t="inlineStr">
+        <is>
+          <t>鳳凰 AI 黃金合約條款 (保命金句)</t>
+        </is>
+      </c>
+      <c r="D3" s="86" t="inlineStr">
+        <is>
+          <t>貴公司現有合約是否具備？</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="100" customHeight="1" s="12">
+      <c r="A4" s="87" t="inlineStr">
+        <is>
+          <t>一、授權範圍與「AI 重製/生成權」雙重分離</t>
+        </is>
+      </c>
+      <c r="B4" s="88" t="inlineStr">
+        <is>
+          <t>「甲方同意無償授權乙方拍攝之照片及影片做為宣傳使用。」
+(風險：同意拍實體片，不代表同意被AI煉丹複製。若無註明AI數位孿生、生成式重製，未來AI生成的影片屬侵權。)</t>
+        </is>
+      </c>
+      <c r="C4" s="88" t="inlineStr">
+        <is>
+          <t>「授權人同意將包含其肖像之影音資料，授權被授權人進行包含但不限於『AI 模型訓練』、『特徵萃取』、『數位分身(Digital Twin)合成』、『語音克隆』等生成式 AI 重製行為，並同意被授權人享有由上述 AI 技術生成之衍生影音作品之完整著作財產權。」</t>
+        </is>
+      </c>
+      <c r="D4" s="87" t="inlineStr"/>
+    </row>
+    <row r="5" ht="100" customHeight="1" s="12">
+      <c r="A5" s="87" t="inlineStr">
+        <is>
+          <t>二、明定「合理對價之買斷性質」</t>
+        </is>
+      </c>
+      <c r="B5" s="88" t="inlineStr">
+        <is>
+          <t>「基於雙方僱傭關係，員工同意無償授權公司使用其肖像...」
+(風險：依據民法，無償贈與可依法撤銷。若無給付對價，員工未來隨時能以侵害人格權為由要求撤回授權。)</t>
+        </is>
+      </c>
+      <c r="C5" s="88" t="inlineStr">
+        <is>
+          <t>「本授權為有償且不可撤回之授權。雙方同意授權對價為新台幣 ____ 元整 (或明定包含於每月薪資之特定加給中)。授權人確認已充分收受該對價，並承諾日後絕不以任何理由撤銷、終止本授權或主張任何額外之權利金。」</t>
+        </is>
+      </c>
+      <c r="D5" s="87" t="inlineStr"/>
+    </row>
+    <row r="6" ht="100" customHeight="1" s="12">
+      <c r="A6" s="87" t="inlineStr">
+        <is>
+          <t>三、僱傭關係終止後之效力豁免</t>
+        </is>
+      </c>
+      <c r="B6" s="88" t="inlineStr">
+        <is>
+          <t>「本同意書於雙方僱傭存續期間有效。」或未約定離職後效力。
+(風險：員工一旦離職，肖像授權自動失效，公司必須將所有含有該員工臉部特徵的 YouTube、官網行銷影片全數下架。)</t>
+        </is>
+      </c>
+      <c r="C6" s="88" t="inlineStr">
+        <is>
+          <t>「本授權之效力不受雙方僱傭關係終止、解除、或變更之影響。授權人離職後，被授權人仍有權永久、不限地域、不限次數，將已生成及未來基於本合約授權生成之 AI 衍生影音內容，用於商業行銷、對外宣傳及所有合法之營運目的。」</t>
+        </is>
+      </c>
+      <c r="D6" s="87" t="inlineStr"/>
+    </row>
+    <row r="8" ht="25" customHeight="1" s="12">
+      <c r="A8" s="89" t="inlineStr">
+        <is>
+          <t>AI 肖像安全度加權分數 (具備保命條款數 / 總條款數)</t>
+        </is>
+      </c>
+      <c r="D8" s="90">
+        <f>COUNTIF(D4:D6, "是 (已包含)") &amp; " / 3"</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D4 D5 D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"是 (已包含),否 (需修改),不適用"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>